<commit_message>
Add diagrams, wireframes, PTR report, and improve startup script
- Add 56 sequence diagrams and 6 combined activity diagrams (Mermaid)
- Add 33 wireframe screenshots for PTR Section 7
- Add Preliminary Technical Report and Demo Q&A docs
- Update start.sh with Redis, Celery, and migration timeout
- Add traffic filter threshold and alert enhancements
- Remove old markdown diagram files (replaced by Mermaid PNGs)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/User Stories Table.xlsx
+++ b/docs/User Stories Table.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="15" customWidth="1" style="9" min="1" max="1"/>
@@ -2311,6 +2311,228 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="14" t="inlineStr">
+        <is>
+          <t>US-51</t>
+        </is>
+      </c>
+      <c r="B52" s="14" t="inlineStr">
+        <is>
+          <t>Free User</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="inlineStr">
+        <is>
+          <t>False Positive Management</t>
+        </is>
+      </c>
+      <c r="D52" s="14" t="inlineStr">
+        <is>
+          <t>As a Free User, I want to add IP addresses to a whitelist to mark false positives, so that trusted IPs are not repeatedly flagged as threats.</t>
+        </is>
+      </c>
+      <c r="E52" s="14" t="inlineStr">
+        <is>
+          <t>WhitelistedIP model, GET/POST /api/alerts/whitelist/, DELETE /api/alerts/whitelist/{id}/</t>
+        </is>
+      </c>
+      <c r="F52" s="14" t="inlineStr">
+        <is>
+          <t>WhitelistPage.jsx (add/remove IPs, reason field)</t>
+        </is>
+      </c>
+      <c r="G52" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="14" t="inlineStr">
+        <is>
+          <t>US-52</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>Premium User</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>Traffic Filter Configuration</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="inlineStr">
+        <is>
+          <t>As a Premium User, I want to configure traffic filter rules with categories, thresholds, and actions, so that the IDS can automatically detect and respond to suspicious traffic patterns.</t>
+        </is>
+      </c>
+      <c r="E53" s="14" t="inlineStr">
+        <is>
+          <t>TrafficFilterRule model, CRUD /api/alerts/traffic-filters/, toggle endpoint</t>
+        </is>
+      </c>
+      <c r="F53" s="14" t="inlineStr">
+        <is>
+          <t>TrafficFilterPage.jsx (rule creation, category/action selectors, toggle)</t>
+        </is>
+      </c>
+      <c r="G53" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="14" t="inlineStr">
+        <is>
+          <t>US-53</t>
+        </is>
+      </c>
+      <c r="B54" s="14" t="inlineStr">
+        <is>
+          <t>Free User</t>
+        </is>
+      </c>
+      <c r="C54" s="14" t="inlineStr">
+        <is>
+          <t>Block Management</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="inlineStr">
+        <is>
+          <t>As a Free User, I want to view a list of all blocked IP addresses and manually unblock them, so that I can manage network access control effectively.</t>
+        </is>
+      </c>
+      <c r="E54" s="14" t="inlineStr">
+        <is>
+          <t>BlockedIP model, GET /api/alerts/blocked-ips/, POST /api/alerts/blocked-ips/{id}/unblock/</t>
+        </is>
+      </c>
+      <c r="F54" s="14" t="inlineStr">
+        <is>
+          <t>BlockedIPsPage.jsx (blocked IP list, search, unblock button)</t>
+        </is>
+      </c>
+      <c r="G54" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="14" t="inlineStr">
+        <is>
+          <t>US-54</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>Premium User</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>Log Ingestion</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="inlineStr">
+        <is>
+          <t>As a Premium User, I want to upload JSON or CSV log files for analysis, so that I can import external log data into the IDS for detection.</t>
+        </is>
+      </c>
+      <c r="E55" s="14" t="inlineStr">
+        <is>
+          <t>LogUpload model, POST /api/alerts/log-upload/, GET /api/alerts/log-upload/history/</t>
+        </is>
+      </c>
+      <c r="F55" s="14" t="inlineStr">
+        <is>
+          <t>LogIngestionPage.jsx (drag-and-drop upload, history table, sample templates)</t>
+        </is>
+      </c>
+      <c r="G55" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="14" t="inlineStr">
+        <is>
+          <t>US-55</t>
+        </is>
+      </c>
+      <c r="B56" s="14" t="inlineStr">
+        <is>
+          <t>Premium User</t>
+        </is>
+      </c>
+      <c r="C56" s="14" t="inlineStr">
+        <is>
+          <t>Visualisation</t>
+        </is>
+      </c>
+      <c r="D56" s="14" t="inlineStr">
+        <is>
+          <t>As a Premium User, I want to create custom visualisations with configurable chart types, axis grouping, breakdown dimensions, and date ranges, so that I can analyse security data in meaningful ways.</t>
+        </is>
+      </c>
+      <c r="E56" s="14" t="inlineStr">
+        <is>
+          <t>GET /api/alerts/analytics/ with group_by, breakdown_by, date_from, date_to params</t>
+        </is>
+      </c>
+      <c r="F56" s="14" t="inlineStr">
+        <is>
+          <t>CustomVisualizationPage.jsx (Line/Bar/Area/Pie, presets, date range pickers)</t>
+        </is>
+      </c>
+      <c r="G56" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="14" t="inlineStr">
+        <is>
+          <t>US-56</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>System Oversight</t>
+        </is>
+      </c>
+      <c r="D57" s="14" t="inlineStr">
+        <is>
+          <t>As an Administrator, I want all admin actions (suspend, unsuspend, reset password, upgrade/downgrade subscription) to be automatically logged in the audit trail, so that administrative changes are fully traceable.</t>
+        </is>
+      </c>
+      <c r="E57" s="14" t="inlineStr">
+        <is>
+          <t>AuditLog.objects.create() in AdminSuspend/Unsuspend/ResetPassword/UpdateSubscription views</t>
+        </is>
+      </c>
+      <c r="F57" s="14" t="inlineStr">
+        <is>
+          <t>Visible in AuditLogsPage.jsx</t>
+        </is>
+      </c>
+      <c r="G57" s="15" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>